<commit_message>
Added .Htaccess and Spicker
</commit_message>
<xml_diff>
--- a/LernplanM293.xlsx
+++ b/LernplanM293.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\staubt\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bwdbern-my.sharepoint.com/personal/leonid_stevanovski_bwdbern_ch/Documents/Desktop/Gibb/M293/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA66B5E-D06E-4FD6-B0F7-98FF894224E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="742" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="742" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Übersicht" sheetId="1" r:id="rId1"/>
@@ -654,7 +654,24 @@
   </cellStyles>
   <dxfs count="25">
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -711,24 +728,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1067,7 +1067,7 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable>
                     <c15:dlblFTEntry>
-                      <c15:txfldGUID>{9FB28BAC-C60B-4A04-B0E2-2CD151EB79D7}</c15:txfldGUID>
+                      <c15:txfldGUID>{ABAA118C-9EAF-43AD-B378-A501A4B09A3C}</c15:txfldGUID>
                       <c15:f>Einstellungen!$F$3</c15:f>
                       <c15:dlblFieldTableCache>
                         <c:ptCount val="1"/>
@@ -1325,7 +1325,7 @@
                   <c:v>45883</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46192</c:v>
+                  <c:v>46260</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>45963</c:v>
@@ -1399,7 +1399,7 @@
                   <c:v>45883</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46192</c:v>
+                  <c:v>46260</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>45963</c:v>
@@ -1417,7 +1417,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>386.25</c:v>
+                  <c:v>471.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>100</c:v>
@@ -1976,7 +1976,7 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable>
                     <c15:dlblFTEntry>
-                      <c15:txfldGUID>{FE8462ED-9247-419B-B132-4791624A4F6A}</c15:txfldGUID>
+                      <c15:txfldGUID>{8BB52AC8-26F6-4576-9D63-21D29D1CA6EB}</c15:txfldGUID>
                       <c15:f>Einstellungen!$F$3</c15:f>
                       <c15:dlblFieldTableCache>
                         <c:ptCount val="1"/>
@@ -2234,7 +2234,7 @@
                   <c:v>45883</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46192</c:v>
+                  <c:v>46260</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>45963</c:v>
@@ -2308,7 +2308,7 @@
                   <c:v>45883</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46192</c:v>
+                  <c:v>46260</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>45963</c:v>
@@ -2326,7 +2326,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>386.25</c:v>
+                  <c:v>471.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>100</c:v>
@@ -4952,18 +4952,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FB8E1E66-9B45-4B11-8B16-1ECFFE0141C6}" name="Tabelle2" displayName="Tabelle2" ref="A3:C5" totalsRowCount="1" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FB8E1E66-9B45-4B11-8B16-1ECFFE0141C6}" name="Tabelle2" displayName="Tabelle2" ref="A3:C5" totalsRowCount="1" headerRowDxfId="5" dataDxfId="4" totalsRowDxfId="3">
   <autoFilter ref="A3:C4" xr:uid="{B4B49017-04D7-48A2-A278-51162B58EE12}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{29A0066F-0408-4E99-A2AE-6392386DCD8D}" name="Thema" totalsRowLabel="Ergebnis" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{F6E30C46-BEE0-4CA5-9718-95D22DB2D380}" name="Erreichte Punkte " totalsRowFunction="sum" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{29A0066F-0408-4E99-A2AE-6392386DCD8D}" name="Thema" totalsRowLabel="Ergebnis" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{F6E30C46-BEE0-4CA5-9718-95D22DB2D380}" name="Erreichte Punkte " totalsRowFunction="sum" dataDxfId="1">
       <calculatedColumnFormula>Workshops!E1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{054F4E7D-B6A2-4809-B0CE-B81EB55497C8}" name="Mögliche Punkte" dataDxfId="19">
+    <tableColumn id="3" xr3:uid="{054F4E7D-B6A2-4809-B0CE-B81EB55497C8}" name="Mögliche Punkte" dataDxfId="0">
       <calculatedColumnFormula>Workshops!D1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4975,8 +4975,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{473475C4-7502-4401-AB8F-B854DC1A24D3}" name="Tabelle1416215" displayName="Tabelle1416215" ref="B62:F63" totalsRowShown="0">
   <autoFilter ref="B62:F63" xr:uid="{473475C4-7502-4401-AB8F-B854DC1A24D3}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{1AD84DC1-279D-4B22-96FF-FBBFC6B69D4B}" name="Ich kann/weiss/habe…" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{3B559249-8019-407D-B22D-40E3360A70D8}" name="Tätigkeitsnachweis" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{1AD84DC1-279D-4B22-96FF-FBBFC6B69D4B}" name="Ich kann/weiss/habe…" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{3B559249-8019-407D-B22D-40E3360A70D8}" name="Tätigkeitsnachweis" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{5AB5D987-E472-43B4-A35F-FB9BDECB7AE3}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{7A921969-BC71-4C43-AEC3-03ED723958DE}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{1C042930-3FFE-49E8-9EEA-77E7ED1AE7EB}" name="Bemerkungen"/>
@@ -4989,8 +4989,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5246F0D4-E28C-409F-A873-021BB04CE176}" name="Tabelle1416186" displayName="Tabelle1416186" ref="B70:F94" totalsRowShown="0">
   <autoFilter ref="B70:F94" xr:uid="{5246F0D4-E28C-409F-A873-021BB04CE176}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{21DBEE18-82C2-41FF-AD6A-67F7D123ECDE}" name="Ich kann/weiss/habe…" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{9108DF69-C6E9-48E4-9B28-BF0900C34C58}" name="Tätigkeitsnachweis" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{21DBEE18-82C2-41FF-AD6A-67F7D123ECDE}" name="Ich kann/weiss/habe…" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{9108DF69-C6E9-48E4-9B28-BF0900C34C58}" name="Tätigkeitsnachweis" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{1CA3AAE8-909B-4BA9-8A95-150D1B630855}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{E5BD24D0-B6AF-4E5C-88DD-49BDA5DC9597}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{CBFCDC16-F8E2-4B90-BD33-61E31BCDBC6D}" name="Bemerkungen"/>
@@ -5009,7 +5009,7 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="2" xr3:uid="{08A0C231-0B4B-4439-9D1F-E98D83825C39}" name="Ich kann/weiss/habe…" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{08A0C231-0B4B-4439-9D1F-E98D83825C39}" name="Ich kann/weiss/habe…" dataDxfId="24"/>
     <tableColumn id="3" xr3:uid="{22E79466-919F-407B-B8E3-37BFB94097F4}" name="Tätigkeitsnachweis"/>
     <tableColumn id="4" xr3:uid="{B1C70E5E-AB95-438C-9C77-C0F6983A28B6}" name="Mögliche Punkte"/>
     <tableColumn id="5" xr3:uid="{4F3D2F03-2CF3-41E3-87BB-C1DCFA400CB0}" name="Erreichte Punkte"/>
@@ -5029,8 +5029,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{CFB4A73D-5305-4682-9318-194DF6303837}" name="Ich kann/weiss/habe…" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{63021F7D-4B98-4B5C-8862-2F09340BF529}" name="Tätigkeitsnachweis" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{CFB4A73D-5305-4682-9318-194DF6303837}" name="Ich kann/weiss/habe…" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{63021F7D-4B98-4B5C-8862-2F09340BF529}" name="Tätigkeitsnachweis" dataDxfId="22"/>
     <tableColumn id="3" xr3:uid="{F2C979FF-6B47-4A39-AD59-1D47227AF95F}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{FB823FE0-FBC0-4209-A33C-8338FE879C69}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{A3FD6BDD-A678-4F8C-A8BE-4D5891BF2F2B}" name="Bemerkungen"/>
@@ -5049,8 +5049,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8EA5AA34-8D15-4BBB-924C-662143577838}" name="Ich kann/weiss/habe…" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{7FFD4647-03CC-472D-82D4-C9BDE4BAB6CB}" name="Tätigkeitsnachweis" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{8EA5AA34-8D15-4BBB-924C-662143577838}" name="Ich kann/weiss/habe…" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{7FFD4647-03CC-472D-82D4-C9BDE4BAB6CB}" name="Tätigkeitsnachweis" dataDxfId="20"/>
     <tableColumn id="3" xr3:uid="{9FACC584-F391-434E-848D-D85A5491FA07}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{FA6AEA62-91D5-4C77-B102-CB1657442291}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{C5521F4A-04FC-4855-8ABE-C329AAD12376}" name="Bemerkungen"/>
@@ -5069,8 +5069,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F0B30DE7-B058-4E90-B220-E17037C30E30}" name="Ich kann/weiss/habe…" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{351FA7DA-7BF5-4F26-AFD7-D0FE92F19F8C}" name="Tätigkeitsnachweis" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{F0B30DE7-B058-4E90-B220-E17037C30E30}" name="Ich kann/weiss/habe…" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{351FA7DA-7BF5-4F26-AFD7-D0FE92F19F8C}" name="Tätigkeitsnachweis" dataDxfId="18"/>
     <tableColumn id="3" xr3:uid="{0B5B8618-920E-457A-B86F-143458131F6C}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{F36D93CA-6241-4C42-91FD-9A12AF3E6165}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{5DAEA38F-A981-43C5-933B-532C25FD0FE5}" name="Bemerkungen"/>
@@ -5089,8 +5089,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7F3E4F11-E6FB-4C95-9925-DCAC233DE551}" name="Ich kann/weiss/habe…" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{763B3FF8-7863-4313-8C4F-7E8D9ABADBDF}" name="Tätigkeitsnachweis" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{7F3E4F11-E6FB-4C95-9925-DCAC233DE551}" name="Ich kann/weiss/habe…" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{763B3FF8-7863-4313-8C4F-7E8D9ABADBDF}" name="Tätigkeitsnachweis" dataDxfId="16"/>
     <tableColumn id="3" xr3:uid="{A083D40A-750D-40EE-B2D5-3F5550091210}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{70B8CA42-0808-4764-A602-0FD47892DE47}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{D20F4EE0-31A8-4B35-95CC-3224E836CF17}" name="Bemerkungen"/>
@@ -5109,8 +5109,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{043E4EFC-5248-419E-AA0A-3BD2A3986270}" name="Ich kann/weiss/habe…" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{05CBD9BF-327E-4EB2-8AAF-CF75E43E82E4}" name="Tätigkeitsnachweis" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{043E4EFC-5248-419E-AA0A-3BD2A3986270}" name="Ich kann/weiss/habe…" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{05CBD9BF-327E-4EB2-8AAF-CF75E43E82E4}" name="Tätigkeitsnachweis" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{7DE6DB28-CC5B-4725-9091-7B6D8472527C}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{7E103BEB-1869-4515-84EF-BC0A4A30CD41}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{5FF02028-21A1-4AF5-9B11-49326B0E2EFF}" name="Bemerkungen"/>
@@ -5129,8 +5129,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{489834AF-5E8B-4EBE-B2A6-4DBFFAB88126}" name="Ich kann/weiss/habe…" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{401C4F57-F8C9-4074-9213-CFE55B345B57}" name="Tätigkeitsnachweis" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{489834AF-5E8B-4EBE-B2A6-4DBFFAB88126}" name="Ich kann/weiss/habe…" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{401C4F57-F8C9-4074-9213-CFE55B345B57}" name="Tätigkeitsnachweis" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{F25A1BB1-73F3-48E7-A2CB-799D76898860}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{D0F26D42-28ED-4180-80CB-9A2AD4067FEA}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{776C1243-8BCF-4893-B9E4-72CA0A6FEF0A}" name="Bemerkungen"/>
@@ -5149,8 +5149,8 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{CCCE29AA-55E1-4B8A-9913-8036861F09C7}" name="Ich kann/weiss/habe…" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{9E452A08-D9DA-4381-B6D6-65C267C5B087}" name="Tätigkeitsnachweis" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{CCCE29AA-55E1-4B8A-9913-8036861F09C7}" name="Ich kann/weiss/habe…" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{9E452A08-D9DA-4381-B6D6-65C267C5B087}" name="Tätigkeitsnachweis" dataDxfId="10"/>
     <tableColumn id="3" xr3:uid="{4FF33111-9D12-47ED-85EA-391262F970A0}" name="Mögliche Punkte"/>
     <tableColumn id="4" xr3:uid="{7CCB66F2-95FC-4CC7-A03C-D4EF2EF8B65F}" name="Erreichte Punkte"/>
     <tableColumn id="6" xr3:uid="{F013C3AF-8A36-49F0-AB5E-5F5B5261255D}" name="Bemerkungen"/>
@@ -5426,19 +5426,19 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="34.26953125" customWidth="1"/>
+    <col min="2" max="2" width="29.26953125" customWidth="1"/>
+    <col min="3" max="3" width="20.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="31.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -5449,7 +5449,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -5460,7 +5460,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -5482,7 +5482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -5490,7 +5490,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>109</v>
       </c>
@@ -5499,7 +5499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="19" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="11" t="s">
         <v>13</v>
       </c>
@@ -5508,16 +5508,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="C10" s="12"/>
     </row>
-    <row r="16" spans="1:5" ht="21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="21" x14ac:dyDescent="0.5">
       <c r="D16" s="13"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="7"/>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="7"/>
     </row>
   </sheetData>
@@ -5536,16 +5536,16 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:F98"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="88.7109375" customWidth="1"/>
-    <col min="3" max="3" width="53.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="88.7265625" customWidth="1"/>
+    <col min="3" max="3" width="53.26953125" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B1" s="6" t="s">
         <v>37</v>
       </c>
@@ -5560,7 +5560,7 @@
       </c>
       <c r="F1" s="6"/>
     </row>
-    <row r="2" spans="1:6" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="19.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B2" s="4" t="s">
         <v>49</v>
       </c>
@@ -5568,7 +5568,7 @@
       <c r="D2" s="15"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="31" t="s">
         <v>0</v>
       </c>
@@ -5585,7 +5585,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B4" s="33" t="s">
         <v>91</v>
       </c>
@@ -5598,7 +5598,7 @@
       <c r="E4" s="33"/>
       <c r="F4" s="33"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="36" t="s">
         <v>69</v>
       </c>
@@ -5609,7 +5609,7 @@
       <c r="E5" s="35"/>
       <c r="F5" s="35"/>
     </row>
-    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A7" s="19" t="s">
         <v>32</v>
       </c>
@@ -5621,7 +5621,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="34"/>
     </row>
-    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="27">
         <v>0.25</v>
       </c>
@@ -5641,7 +5641,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="20"/>
       <c r="B9" s="1" t="s">
         <v>70</v>
@@ -5650,7 +5650,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="20"/>
       <c r="B10" t="s">
         <v>71</v>
@@ -5659,14 +5659,14 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="20"/>
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="20"/>
     </row>
-    <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A13" s="20"/>
       <c r="B13" s="4" t="s">
         <v>29</v>
@@ -5676,7 +5676,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="34"/>
     </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="20"/>
       <c r="B14" t="s">
         <v>0</v>
@@ -5694,7 +5694,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="20"/>
       <c r="B15" t="s">
         <v>72</v>
@@ -5703,7 +5703,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="20"/>
       <c r="B16" t="s">
         <v>73</v>
@@ -5712,7 +5712,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="20"/>
       <c r="B17" s="1" t="s">
         <v>42</v>
@@ -5721,7 +5721,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="20"/>
       <c r="B18" s="1" t="s">
         <v>43</v>
@@ -5730,7 +5730,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="20"/>
       <c r="B19" s="1" t="s">
         <v>44</v>
@@ -5739,7 +5739,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="20"/>
       <c r="B20" s="1" t="s">
         <v>57</v>
@@ -5749,7 +5749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="20"/>
       <c r="B21" s="1" t="s">
         <v>58</v>
@@ -5759,7 +5759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="20"/>
       <c r="B22" s="1" t="s">
         <v>59</v>
@@ -5769,7 +5769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="20"/>
       <c r="B23" s="1" t="s">
         <v>60</v>
@@ -5779,7 +5779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="20"/>
       <c r="B24" s="1" t="s">
         <v>61</v>
@@ -5789,10 +5789,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="20"/>
     </row>
-    <row r="26" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A26" s="20"/>
       <c r="B26" s="4" t="s">
         <v>30</v>
@@ -5804,7 +5804,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="20"/>
       <c r="B27" t="s">
         <v>0</v>
@@ -5822,7 +5822,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="20"/>
       <c r="B28" s="1" t="s">
         <v>102</v>
@@ -5834,7 +5834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="20"/>
       <c r="B29" s="1" t="s">
         <v>103</v>
@@ -5846,7 +5846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="20"/>
       <c r="B30" s="1" t="s">
         <v>104</v>
@@ -5858,10 +5858,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="20"/>
     </row>
-    <row r="32" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A32" s="20"/>
       <c r="B32" s="4" t="s">
         <v>98</v>
@@ -5873,7 +5873,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="20"/>
       <c r="B33" t="s">
         <v>0</v>
@@ -5891,14 +5891,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="20"/>
       <c r="B34" t="s">
         <v>45</v>
       </c>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="20"/>
       <c r="B35" s="1" t="s">
         <v>105</v>
@@ -5910,10 +5910,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="20"/>
     </row>
-    <row r="37" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A37" s="20"/>
       <c r="B37" s="4" t="s">
         <v>99</v>
@@ -5922,7 +5922,7 @@
       <c r="D37" s="17"/>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="20"/>
       <c r="B38" t="s">
         <v>0</v>
@@ -5940,17 +5940,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="20"/>
       <c r="B39" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C39" s="1"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="20"/>
     </row>
-    <row r="41" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A41" s="20"/>
       <c r="B41" s="4" t="s">
         <v>31</v>
@@ -5962,7 +5962,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A42" s="20"/>
       <c r="B42" t="s">
         <v>0</v>
@@ -5980,7 +5980,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="20"/>
       <c r="B43" t="s">
         <v>92</v>
@@ -5992,11 +5992,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="20"/>
       <c r="C44" s="1"/>
     </row>
-    <row r="45" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A45" s="20"/>
       <c r="B45" s="5" t="s">
         <v>34</v>
@@ -6012,8 +6012,8 @@
       </c>
       <c r="F45" s="6"/>
     </row>
-    <row r="46" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="47" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A47" s="22" t="s">
         <v>33</v>
       </c>
@@ -6027,7 +6027,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="26">
         <v>0.25</v>
       </c>
@@ -6047,7 +6047,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="21"/>
       <c r="B49" s="1" t="s">
         <v>106</v>
@@ -6060,7 +6060,7 @@
       </c>
       <c r="E49" s="1"/>
     </row>
-    <row r="50" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="21"/>
       <c r="B50" s="1" t="s">
         <v>107</v>
@@ -6072,10 +6072,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="21"/>
     </row>
-    <row r="52" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A52" s="21"/>
       <c r="B52" s="4" t="s">
         <v>101</v>
@@ -6086,7 +6086,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="21"/>
       <c r="B53" t="s">
         <v>0</v>
@@ -6104,7 +6104,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="21"/>
       <c r="B54" s="1" t="s">
         <v>108</v>
@@ -6117,7 +6117,7 @@
       </c>
       <c r="E54" s="1"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="21"/>
       <c r="B55" s="1" t="s">
         <v>47</v>
@@ -6130,7 +6130,7 @@
       </c>
       <c r="E55" s="1"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="21"/>
       <c r="B56" s="1" t="s">
         <v>40</v>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="E56" s="1"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="21"/>
       <c r="B57" s="1" t="s">
         <v>93</v>
@@ -6156,7 +6156,7 @@
       </c>
       <c r="E57" s="1"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="21"/>
       <c r="B58" s="1" t="s">
         <v>56</v>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="E58" s="1"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="21"/>
       <c r="B59" s="1" t="s">
         <v>48</v>
@@ -6182,10 +6182,10 @@
       </c>
       <c r="E59" s="1"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="21"/>
     </row>
-    <row r="61" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A61" s="21"/>
       <c r="B61" s="4" t="s">
         <v>35</v>
@@ -6196,7 +6196,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A62" s="21"/>
       <c r="B62" t="s">
         <v>0</v>
@@ -6214,7 +6214,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="21"/>
       <c r="B63" t="s">
         <v>94</v>
@@ -6226,18 +6226,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="21"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="21"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="21"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
     </row>
-    <row r="67" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A67" s="21"/>
       <c r="B67" s="5" t="s">
         <v>4</v>
@@ -6253,8 +6253,8 @@
       </c>
       <c r="F67" s="6"/>
     </row>
-    <row r="68" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="69" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A69" s="23" t="s">
         <v>36</v>
       </c>
@@ -6268,7 +6268,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A70" s="25">
         <v>0.5</v>
       </c>
@@ -6288,7 +6288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A71" s="24"/>
       <c r="B71" s="1" t="s">
         <v>74</v>
@@ -6297,7 +6297,7 @@
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
     </row>
-    <row r="72" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="24"/>
       <c r="B72" s="29" t="s">
         <v>63</v>
@@ -6306,7 +6306,7 @@
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
     </row>
-    <row r="73" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="24"/>
       <c r="B73" s="1" t="s">
         <v>55</v>
@@ -6315,7 +6315,7 @@
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="24"/>
       <c r="B74" s="1" t="s">
         <v>75</v>
@@ -6326,7 +6326,7 @@
       </c>
       <c r="E74" s="1"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="24"/>
       <c r="B75" s="1" t="s">
         <v>76</v>
@@ -6337,7 +6337,7 @@
       </c>
       <c r="E75" s="1"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="24"/>
       <c r="B76" s="1" t="s">
         <v>77</v>
@@ -6348,7 +6348,7 @@
       </c>
       <c r="E76" s="1"/>
     </row>
-    <row r="77" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="24"/>
       <c r="B77" s="1" t="s">
         <v>78</v>
@@ -6361,14 +6361,14 @@
       </c>
       <c r="E77" s="1"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="24"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
     </row>
-    <row r="79" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="24"/>
       <c r="B79" s="1" t="s">
         <v>86</v>
@@ -6377,7 +6377,7 @@
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
     </row>
-    <row r="80" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="24"/>
       <c r="B80" s="37" t="s">
         <v>65</v>
@@ -6387,7 +6387,7 @@
       </c>
       <c r="E80" s="1"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="24"/>
       <c r="B81" s="1" t="s">
         <v>52</v>
@@ -6397,7 +6397,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="24"/>
       <c r="B82" s="1" t="s">
         <v>95</v>
@@ -6407,7 +6407,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="24"/>
       <c r="B83" s="1" t="s">
         <v>79</v>
@@ -6417,7 +6417,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="24"/>
       <c r="B84" s="1" t="s">
         <v>80</v>
@@ -6427,7 +6427,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="24"/>
       <c r="B85" s="1" t="s">
         <v>81</v>
@@ -6437,7 +6437,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="24"/>
       <c r="B86" s="1" t="s">
         <v>88</v>
@@ -6447,7 +6447,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="24"/>
       <c r="B87" s="1" t="s">
         <v>82</v>
@@ -6457,7 +6457,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="24"/>
       <c r="B88" s="1" t="s">
         <v>83</v>
@@ -6467,7 +6467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="24"/>
       <c r="B89" s="1" t="s">
         <v>84</v>
@@ -6477,7 +6477,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="24"/>
       <c r="B90" s="1" t="s">
         <v>85</v>
@@ -6487,7 +6487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="24"/>
       <c r="B91" s="1" t="s">
         <v>89</v>
@@ -6497,7 +6497,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="24"/>
       <c r="B92" s="1" t="s">
         <v>64</v>
@@ -6507,7 +6507,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="24"/>
       <c r="B93" s="1" t="s">
         <v>54</v>
@@ -6517,18 +6517,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="24"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="24"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="24"/>
     </row>
-    <row r="97" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" ht="19" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A97" s="24"/>
       <c r="B97" s="5" t="s">
         <v>4</v>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="F97" s="6"/>
     </row>
-    <row r="98" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -6566,14 +6566,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B9E32F-A66D-4D86-8DDB-1A02024B176D}">
   <dimension ref="B2:N33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>15</v>
       </c>
@@ -6581,7 +6581,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>14</v>
       </c>
@@ -6596,7 +6596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>17</v>
       </c>
@@ -6610,7 +6610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>18</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>19</v>
       </c>
@@ -6632,7 +6632,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>20</v>
       </c>
@@ -6640,7 +6640,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>24</v>
       </c>
@@ -6655,13 +6655,13 @@
       </c>
       <c r="N9" s="9"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="7">
         <f ca="1">TODAY()</f>
-        <v>46192</v>
+        <v>46260</v>
       </c>
       <c r="D10">
         <f>F3</f>
@@ -6669,10 +6669,10 @@
       </c>
       <c r="E10">
         <f ca="1">(100*D15)/D13</f>
-        <v>386.25</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+        <v>471.25</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>23</v>
       </c>
@@ -6686,7 +6686,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>96</v>
       </c>
@@ -6695,7 +6695,7 @@
         <v>45923</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>25</v>
       </c>
@@ -6704,7 +6704,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>26</v>
       </c>
@@ -6713,31 +6713,31 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>97</v>
       </c>
       <c r="D15">
         <f ca="1">DATEDIF(C9,C10,"d")</f>
-        <v>309</v>
-      </c>
-    </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="29" spans="3:4" x14ac:dyDescent="0.35">
       <c r="D29" s="8"/>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
     </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
     </row>

</xml_diff>